<commit_message>
changed url in backend
</commit_message>
<xml_diff>
--- a/backend/ad_stats_log.xlsx
+++ b/backend/ad_stats_log.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F372"/>
+  <dimension ref="A1:F385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27.28515625" customWidth="1" min="1" max="1"/>
@@ -8708,6 +8708,227 @@
         </is>
       </c>
     </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:35:10</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:35:11</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:35:12</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:35:37</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:35:38</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:35:40</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:35:51</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:40:43</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:40:43</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:41:38</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:41:39</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:41:51</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2025-09-01 14:42:48</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Young Adult (20-34)</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Man</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>